<commit_message>
261008 Fix lỗi lệch tâm điểm gốc cho mã hàng 23691084-260904-inner-nta
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/gateway/products/23691084-260904-inner-nta/23691084-260904-inner-nta.xlsx
+++ b/modules/gateway/products/23691084-260904-inner-nta/23691084-260904-inner-nta.xlsx
@@ -1,21 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Camera\Dev\Service_Manager\modules\gateway\products\23691084-260904-inner-nta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E50B2230-18E6-4CD4-A114-BEC53776F11F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDC942B2-A6AC-4C6D-9244-70BD75784A24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2040" yWindow="1944" windowWidth="17280" windowHeight="10296" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="13464" windowHeight="10296" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calibration_Data" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -74,7 +87,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -98,13 +111,6 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -160,7 +166,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -174,8 +180,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -487,7 +496,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -495,29 +504,29 @@
     <col min="4" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -539,8 +548,9 @@
       <c r="G4" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I4" s="6"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>9</v>
       </c>
@@ -550,20 +560,20 @@
       <c r="C5" s="4">
         <v>25</v>
       </c>
-      <c r="D5" s="4">
-        <v>18.466335999999998</v>
-      </c>
-      <c r="E5" s="4">
-        <v>593.89499999999998</v>
-      </c>
-      <c r="F5" s="4">
-        <v>18.579999999999998</v>
-      </c>
-      <c r="G5" s="4">
-        <v>5.92279</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D5" s="5">
+        <v>416.86234000000002</v>
+      </c>
+      <c r="E5" s="5">
+        <v>40.533000000000001</v>
+      </c>
+      <c r="F5" s="5">
+        <v>416.46034400000002</v>
+      </c>
+      <c r="G5" s="5">
+        <v>628.649</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>10</v>
       </c>
@@ -573,20 +583,20 @@
       <c r="C6" s="4">
         <v>25</v>
       </c>
-      <c r="D6" s="4">
-        <v>17.974</v>
-      </c>
-      <c r="E6" s="4">
-        <v>5.6181049999999999</v>
-      </c>
-      <c r="F6" s="4">
-        <v>17.547999999999998</v>
-      </c>
-      <c r="G6" s="4">
-        <v>594.23834299999999</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D6" s="5">
+        <v>417.20233999999999</v>
+      </c>
+      <c r="E6" s="5">
+        <v>628.87199999999996</v>
+      </c>
+      <c r="F6" s="5">
+        <v>417.58199999999999</v>
+      </c>
+      <c r="G6" s="5">
+        <v>40.305684999999997</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>11</v>
       </c>
@@ -597,19 +607,19 @@
         <v>374</v>
       </c>
       <c r="D7" s="5">
-        <v>367.16699999999997</v>
+        <v>67.944999999999993</v>
       </c>
       <c r="E7" s="5">
-        <v>6.3473430000000004</v>
-      </c>
-      <c r="F7" s="4">
-        <v>366.78201300000001</v>
-      </c>
-      <c r="G7" s="4">
-        <v>595.78855199999998</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+        <v>628.08686699999998</v>
+      </c>
+      <c r="F7" s="5">
+        <v>68.310323999999994</v>
+      </c>
+      <c r="G7" s="5">
+        <v>38.627000000000002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>12</v>
       </c>
@@ -619,20 +629,20 @@
       <c r="C8" s="4">
         <v>377</v>
       </c>
-      <c r="D8" s="4">
-        <v>370.67600399999998</v>
-      </c>
-      <c r="E8" s="4">
-        <v>594.61699999999996</v>
-      </c>
-      <c r="F8" s="4">
-        <v>370.81167199999999</v>
-      </c>
-      <c r="G8" s="4">
-        <v>7.5789999999999997</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D8" s="5">
+        <v>64.635999999999996</v>
+      </c>
+      <c r="E8" s="5">
+        <v>39.705579999999998</v>
+      </c>
+      <c r="F8" s="5">
+        <v>64.187331999999998</v>
+      </c>
+      <c r="G8" s="5">
+        <v>626.99199999999996</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>13</v>
       </c>
@@ -642,20 +652,20 @@
       <c r="C9" s="4">
         <v>8.5</v>
       </c>
-      <c r="D9" s="4">
-        <v>1.865378</v>
-      </c>
-      <c r="E9" s="4">
-        <v>525.26704900000004</v>
-      </c>
-      <c r="F9" s="4">
-        <v>1.9560040000000001</v>
-      </c>
-      <c r="G9" s="4">
-        <v>74.421000000000006</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D9" s="5">
+        <v>433.41300000000001</v>
+      </c>
+      <c r="E9" s="5">
+        <v>109.134343</v>
+      </c>
+      <c r="F9" s="5">
+        <v>433.101</v>
+      </c>
+      <c r="G9" s="5">
+        <v>560.14510499999994</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>14</v>
       </c>
@@ -665,29 +675,29 @@
       <c r="C10" s="4">
         <v>393.5</v>
       </c>
-      <c r="D10" s="4">
-        <v>386.77167200000002</v>
-      </c>
-      <c r="E10" s="4">
-        <v>65.878</v>
-      </c>
-      <c r="F10" s="4">
-        <v>386.37700799999999</v>
-      </c>
-      <c r="G10" s="4">
-        <v>536.47</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="9" t="s">
+      <c r="D10" s="5">
+        <v>48.364986999999999</v>
+      </c>
+      <c r="E10" s="5">
+        <v>568.55899999999997</v>
+      </c>
+      <c r="F10" s="5">
+        <v>48.706656000000002</v>
+      </c>
+      <c r="G10" s="5">
+        <v>98.010999999999996</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>